<commit_message>
Read the supplementary data files directly and load saved results by default
The notebooks now read Supplementary Data 3 and 4 (the Bar orientation of the
balanced designs is stored in (-pi/2, pi/2] in the data file, so no angle
pre-processing is needed), get a RETRAIN switch that loads the saved tables and
models unless retraining is requested, draw figures without writing files, and
use one shared figure style. Supplementary Data 4 gains a sheet with the Pareto
sets of the three confidence levels.
</commit_message>
<xml_diff>
--- a/data/Supplementary Data 4.xlsx
+++ b/data/Supplementary Data 4.xlsx
@@ -17,6 +17,7 @@
     <sheet name="1 Bar-dominant" sheetId="7" r:id="rId2"/>
     <sheet name="2 Balanced" sheetId="5" r:id="rId3"/>
     <sheet name="3 Y-dominant" sheetId="6" r:id="rId4"/>
+    <sheet name="Pareto sets" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3872,7 +3873,7 @@
         <v>1.0659000000000001</v>
       </c>
       <c r="G2" s="3">
-        <v>2.8940000000000001</v>
+        <v>-0.247592653589793</v>
       </c>
       <c r="H2" s="3">
         <v>1.365</v>
@@ -3898,7 +3899,7 @@
         <v>1.0924999999999998</v>
       </c>
       <c r="G3" s="3">
-        <v>2.919</v>
+        <v>-0.22259265358979308</v>
       </c>
       <c r="H3" s="3">
         <v>1.4019999999999999</v>
@@ -3924,7 +3925,7 @@
         <v>1.1148</v>
       </c>
       <c r="G4" s="3">
-        <v>2.8980000000000001</v>
+        <v>-0.24359265358979298</v>
       </c>
       <c r="H4" s="3">
         <v>1.405</v>
@@ -3950,7 +3951,7 @@
         <v>1.1184000000000001</v>
       </c>
       <c r="G5" s="3">
-        <v>2.8969999999999998</v>
+        <v>-0.24459265358979332</v>
       </c>
       <c r="H5" s="3">
         <v>1.363</v>
@@ -3976,7 +3977,7 @@
         <v>1.145</v>
       </c>
       <c r="G6" s="3">
-        <v>2.931</v>
+        <v>-0.21059265358979307</v>
       </c>
       <c r="H6" s="3">
         <v>1.407</v>
@@ -4002,7 +4003,7 @@
         <v>1.1674</v>
       </c>
       <c r="G7" s="3">
-        <v>2.9159999999999999</v>
+        <v>-0.2255926535897932</v>
       </c>
       <c r="H7" s="3">
         <v>1.413</v>
@@ -4028,7 +4029,7 @@
         <v>1.1700000000000002</v>
       </c>
       <c r="G8" s="3">
-        <v>2.8969999999999998</v>
+        <v>-0.24459265358979332</v>
       </c>
       <c r="H8" s="3">
         <v>1.361</v>
@@ -4054,7 +4055,7 @@
         <v>1.1988000000000001</v>
       </c>
       <c r="G9" s="3">
-        <v>2.9409999999999998</v>
+        <v>-0.20059265358979328</v>
       </c>
       <c r="H9" s="3">
         <v>1.411</v>
@@ -4080,7 +4081,7 @@
         <v>1.2222</v>
       </c>
       <c r="G10" s="3">
-        <v>2.9329999999999998</v>
+        <v>-0.2085926535897933</v>
       </c>
       <c r="H10" s="3">
         <v>1.421</v>
@@ -4106,7 +4107,7 @@
         <v>1.2222</v>
       </c>
       <c r="G11" s="3">
-        <v>2.8929999999999998</v>
+        <v>-0.24859265358979332</v>
       </c>
       <c r="H11" s="3">
         <v>1.355</v>
@@ -4132,7 +4133,7 @@
         <v>1.2499</v>
       </c>
       <c r="G12" s="3">
-        <v>2.9489999999999998</v>
+        <v>-0.19259265358979327</v>
       </c>
       <c r="H12" s="3">
         <v>1.4139999999999999</v>
@@ -4158,7 +4159,7 @@
         <v>1.2749999999999999</v>
       </c>
       <c r="G13" s="3">
-        <v>2.9470000000000001</v>
+        <v>-0.19459265358979305</v>
       </c>
       <c r="H13" s="3">
         <v>1.427</v>
@@ -4184,7 +4185,7 @@
         <v>1.2734999999999999</v>
       </c>
       <c r="G14" s="3">
-        <v>2.8879999999999999</v>
+        <v>-0.2535926535897932</v>
       </c>
       <c r="H14" s="3">
         <v>1.349</v>
@@ -4210,7 +4211,7 @@
         <v>1.30355</v>
       </c>
       <c r="G15" s="3">
-        <v>2.9550000000000001</v>
+        <v>-0.18659265358979304</v>
       </c>
       <c r="H15" s="3">
         <v>1.4159999999999999</v>
@@ -4236,7 +4237,7 @@
         <v>1.3280000000000001</v>
       </c>
       <c r="G16" s="3">
-        <v>2.9590000000000001</v>
+        <v>-0.18259265358979304</v>
       </c>
       <c r="H16" s="3">
         <v>1.4330000000000001</v>
@@ -4262,7 +4263,7 @@
         <v>1.3360000000000001</v>
       </c>
       <c r="G17" s="3">
-        <v>2.875</v>
+        <v>-0.2665926535897931</v>
       </c>
       <c r="H17" s="3">
         <v>1.34</v>
@@ -4288,7 +4289,7 @@
         <v>1.3562999999999998</v>
       </c>
       <c r="G18" s="3">
-        <v>2.9590000000000001</v>
+        <v>-0.18259265358979304</v>
       </c>
       <c r="H18" s="3">
         <v>1.417</v>
@@ -4314,7 +4315,7 @@
         <v>1.3820999999999999</v>
       </c>
       <c r="G19" s="3">
-        <v>2.968</v>
+        <v>-0.17359265358979314</v>
       </c>
       <c r="H19" s="3">
         <v>1.4370000000000001</v>
@@ -4340,7 +4341,7 @@
         <v>1.4244999999999999</v>
       </c>
       <c r="G20" s="3">
-        <v>2.9209999999999998</v>
+        <v>-0.2205926535897933</v>
       </c>
       <c r="H20" s="3">
         <v>1.4019999999999999</v>
@@ -4366,7 +4367,7 @@
         <v>1.4518925600000001</v>
       </c>
       <c r="G21" s="3">
-        <v>2.8328047600000001</v>
+        <v>-0.30878789358979297</v>
       </c>
       <c r="H21" s="3">
         <v>1.3441136300000001</v>
@@ -4392,7 +4393,7 @@
         <v>1.407</v>
       </c>
       <c r="G22" s="3">
-        <v>2.9620000000000002</v>
+        <v>-0.17959265358979293</v>
       </c>
       <c r="H22" s="3">
         <v>1.417</v>
@@ -4418,7 +4419,7 @@
         <v>1.4346000000000001</v>
       </c>
       <c r="G23" s="3">
-        <v>2.976</v>
+        <v>-0.16559265358979314</v>
       </c>
       <c r="H23" s="3">
         <v>1.44</v>
@@ -4444,7 +4445,7 @@
         <v>1.4578000000000002</v>
       </c>
       <c r="G24" s="3">
-        <v>2.956</v>
+        <v>-0.18559265358979316</v>
       </c>
       <c r="H24" s="3">
         <v>1.4370000000000001</v>
@@ -4470,7 +4471,7 @@
         <v>1.4596500000000001</v>
       </c>
       <c r="G25" s="3">
-        <v>2.9630000000000001</v>
+        <v>-0.17859265358979304</v>
       </c>
       <c r="H25" s="3">
         <v>1.4159999999999999</v>
@@ -4496,7 +4497,7 @@
         <v>1.4896</v>
       </c>
       <c r="G26" s="3">
-        <v>2.9830000000000001</v>
+        <v>-0.15859265358979302</v>
       </c>
       <c r="H26" s="3">
         <v>1.444</v>
@@ -4522,7 +4523,7 @@
         <v>1.51125</v>
       </c>
       <c r="G27" s="3">
-        <v>2.9689999999999999</v>
+        <v>-0.17259265358979325</v>
       </c>
       <c r="H27" s="3">
         <v>1.444</v>
@@ -4548,7 +4549,7 @@
         <v>1.51125</v>
       </c>
       <c r="G28" s="3">
-        <v>2.9620000000000002</v>
+        <v>-0.17959265358979293</v>
       </c>
       <c r="H28" s="3">
         <v>1.413</v>
@@ -4574,7 +4575,7 @@
         <v>1.542</v>
       </c>
       <c r="G29" s="3">
-        <v>2.988</v>
+        <v>-0.15359265358979313</v>
       </c>
       <c r="H29" s="3">
         <v>1.446</v>
@@ -4600,7 +4601,7 @@
         <v>1.5661999999999998</v>
       </c>
       <c r="G30" s="3">
-        <v>2.98</v>
+        <v>-0.16159265358979313</v>
       </c>
       <c r="H30" s="3">
         <v>1.45</v>
@@ -4626,7 +4627,7 @@
         <v>1.5641499999999999</v>
       </c>
       <c r="G31" s="3">
-        <v>2.9569999999999999</v>
+        <v>-0.18459265358979327</v>
       </c>
       <c r="H31" s="3">
         <v>1.4079999999999999</v>
@@ -4652,7 +4653,7 @@
         <v>1.5939000000000001</v>
       </c>
       <c r="G32" s="3">
-        <v>2.9929999999999999</v>
+        <v>-0.14859265358979323</v>
       </c>
       <c r="H32" s="3">
         <v>1.4470000000000001</v>
@@ -4678,7 +4679,7 @@
         <v>1.6189499999999999</v>
       </c>
       <c r="G33" s="3">
-        <v>2.99</v>
+        <v>-0.1515926535897929</v>
       </c>
       <c r="H33" s="3">
         <v>1.456</v>
@@ -4704,7 +4705,7 @@
         <v>1.6146499999999999</v>
       </c>
       <c r="G34" s="3">
-        <v>2.952</v>
+        <v>-0.18959265358979316</v>
       </c>
       <c r="H34" s="3">
         <v>1.4019999999999999</v>
@@ -4730,7 +4731,7 @@
         <v>1.6478000000000002</v>
       </c>
       <c r="G35" s="3">
-        <v>2.9969999999999999</v>
+        <v>-0.14459265358979323</v>
       </c>
       <c r="H35" s="3">
         <v>1.4490000000000001</v>
@@ -4756,7 +4757,7 @@
         <v>1.6739999999999999</v>
       </c>
       <c r="G36" s="3">
-        <v>2.9980000000000002</v>
+        <v>-0.1435926535897929</v>
       </c>
       <c r="H36" s="3">
         <v>1.4590000000000001</v>
@@ -5636,4 +5637,3885 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I121"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <t>κ</t>
+          </r>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <t>Confidence level Φ(κ)</t>
+          </r>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <t>L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+              <sz val="12"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t>0,Bar</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="12"/>
+              <color indexed="8"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve"> [cm]</t>
+          </r>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <t>L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+              <sz val="12"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t>0,Y</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="12"/>
+              <color indexed="8"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve"> [cm]</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <t>Configuration type</t>
+          </r>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <t>Predicted strength [N/m]</t>
+          </r>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <t>σ</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+              <sz val="12"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t>cal</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="12"/>
+              <color indexed="8"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve"> strength [N/m]</t>
+          </r>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <t>Predicted toughness [J/m2]</t>
+          </r>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <t>σ</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+              <sz val="12"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t>cal</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="12"/>
+              <color indexed="8"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve"> toughness [J/m2]</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2.12</v>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F2" s="3">
+        <v>102.803</v>
+      </c>
+      <c r="G2" s="3">
+        <v>4.622</v>
+      </c>
+      <c r="H2" s="3">
+        <v>5.109</v>
+      </c>
+      <c r="I2" s="3">
+        <v>2.065</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D3" s="3">
+        <v>2.12</v>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F3" s="3">
+        <v>102.552</v>
+      </c>
+      <c r="G3" s="3">
+        <v>4.469</v>
+      </c>
+      <c r="H3" s="3">
+        <v>5.138</v>
+      </c>
+      <c r="I3" s="3">
+        <v>2.224</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B4" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F4" s="3">
+        <v>102.28</v>
+      </c>
+      <c r="G4" s="3">
+        <v>5.528</v>
+      </c>
+      <c r="H4" s="3">
+        <v>5.413</v>
+      </c>
+      <c r="I4" s="3">
+        <v>2.65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F5" s="3">
+        <v>102.048</v>
+      </c>
+      <c r="G5" s="3">
+        <v>5.762</v>
+      </c>
+      <c r="H5" s="3">
+        <v>5.462</v>
+      </c>
+      <c r="I5" s="3">
+        <v>2.74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B6" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F6" s="3">
+        <v>101.594</v>
+      </c>
+      <c r="G6" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>5.562</v>
+      </c>
+      <c r="I6" s="3">
+        <v>2.842</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B7" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C7" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D7" s="3">
+        <v>2.08</v>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F7" s="3">
+        <v>101.46</v>
+      </c>
+      <c r="G7" s="3">
+        <v>7.606</v>
+      </c>
+      <c r="H7" s="3">
+        <v>5.757</v>
+      </c>
+      <c r="I7" s="3">
+        <v>3.108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B8" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C8" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D8" s="3">
+        <v>2.08</v>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F8" s="3">
+        <v>101.074</v>
+      </c>
+      <c r="G8" s="3">
+        <v>7.792</v>
+      </c>
+      <c r="H8" s="3">
+        <v>5.851</v>
+      </c>
+      <c r="I8" s="3">
+        <v>3.176</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B9" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>2.06</v>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F9" s="3">
+        <v>100.742</v>
+      </c>
+      <c r="G9" s="3">
+        <v>8.866</v>
+      </c>
+      <c r="H9" s="3">
+        <v>6.064</v>
+      </c>
+      <c r="I9" s="3">
+        <v>3.321</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B10" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C10" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D10" s="3">
+        <v>2.06</v>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F10" s="3">
+        <v>100.143</v>
+      </c>
+      <c r="G10" s="3">
+        <v>8.977</v>
+      </c>
+      <c r="H10" s="3">
+        <v>6.241</v>
+      </c>
+      <c r="I10" s="3">
+        <v>3.342</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D11" s="3">
+        <v>2.04</v>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F11" s="3">
+        <v>99.913</v>
+      </c>
+      <c r="G11" s="3">
+        <v>9.642</v>
+      </c>
+      <c r="H11" s="3">
+        <v>6.458</v>
+      </c>
+      <c r="I11" s="3">
+        <v>3.386</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B12" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C12" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D12" s="3">
+        <v>2.06</v>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F12" s="3">
+        <v>99.133</v>
+      </c>
+      <c r="G12" s="3">
+        <v>9.1</v>
+      </c>
+      <c r="H12" s="3">
+        <v>6.578</v>
+      </c>
+      <c r="I12" s="3">
+        <v>3.337</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B13" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C13" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D13" s="3">
+        <v>2.04</v>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F13" s="3">
+        <v>98.925</v>
+      </c>
+      <c r="G13" s="3">
+        <v>9.744</v>
+      </c>
+      <c r="H13" s="3">
+        <v>6.843</v>
+      </c>
+      <c r="I13" s="3">
+        <v>3.378</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B14" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C14" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>2.02</v>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F14" s="3">
+        <v>98.666</v>
+      </c>
+      <c r="G14" s="3">
+        <v>10.157</v>
+      </c>
+      <c r="H14" s="3">
+        <v>7.182</v>
+      </c>
+      <c r="I14" s="3">
+        <v>3.484</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B15" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C15" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D15" s="3">
+        <v>2.06</v>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F15" s="3">
+        <v>97.448</v>
+      </c>
+      <c r="G15" s="3">
+        <v>9.3</v>
+      </c>
+      <c r="H15" s="3">
+        <v>7.216</v>
+      </c>
+      <c r="I15" s="3">
+        <v>3.302</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B16" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C16" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D16" s="3">
+        <v>2.04</v>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F16" s="3">
+        <v>97.271</v>
+      </c>
+      <c r="G16" s="3">
+        <v>9.933</v>
+      </c>
+      <c r="H16" s="3">
+        <v>7.537</v>
+      </c>
+      <c r="I16" s="3">
+        <v>3.363</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B17" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C17" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D17" s="3">
+        <v>2.02</v>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F17" s="3">
+        <v>96.993</v>
+      </c>
+      <c r="G17" s="3">
+        <v>10.404</v>
+      </c>
+      <c r="H17" s="3">
+        <v>7.94</v>
+      </c>
+      <c r="I17" s="3">
+        <v>3.519</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B18" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C18" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F18" s="3">
+        <v>96.57</v>
+      </c>
+      <c r="G18" s="3">
+        <v>10.914</v>
+      </c>
+      <c r="H18" s="3">
+        <v>8.412</v>
+      </c>
+      <c r="I18" s="3">
+        <v>3.755</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B19" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C19" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D19" s="3">
+        <v>2.04</v>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F19" s="3">
+        <v>94.494</v>
+      </c>
+      <c r="G19" s="3">
+        <v>10.343</v>
+      </c>
+      <c r="H19" s="3">
+        <v>8.74</v>
+      </c>
+      <c r="I19" s="3">
+        <v>3.355</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B20" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C20" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D20" s="3">
+        <v>2.02</v>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F20" s="3">
+        <v>94.233</v>
+      </c>
+      <c r="G20" s="3">
+        <v>10.899</v>
+      </c>
+      <c r="H20" s="3">
+        <v>9.176</v>
+      </c>
+      <c r="I20" s="3">
+        <v>3.555</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B21" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C21" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D21" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F21" s="3">
+        <v>93.759</v>
+      </c>
+      <c r="G21" s="3">
+        <v>11.553</v>
+      </c>
+      <c r="H21" s="3">
+        <v>9.669</v>
+      </c>
+      <c r="I21" s="3">
+        <v>3.797</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B22" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C22" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D22" s="3">
+        <v>1.98</v>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F22" s="3">
+        <v>92.876</v>
+      </c>
+      <c r="G22" s="3">
+        <v>12.519</v>
+      </c>
+      <c r="H22" s="3">
+        <v>10.167</v>
+      </c>
+      <c r="I22" s="3">
+        <v>3.986</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B23" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C23" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D23" s="3">
+        <v>2.04</v>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F23" s="3">
+        <v>89.78</v>
+      </c>
+      <c r="G23" s="3">
+        <v>11.024</v>
+      </c>
+      <c r="H23" s="3">
+        <v>10.696</v>
+      </c>
+      <c r="I23" s="3">
+        <v>3.389</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B24" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C24" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D24" s="3">
+        <v>2.02</v>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F24" s="3">
+        <v>89.598</v>
+      </c>
+      <c r="G24" s="3">
+        <v>11.613</v>
+      </c>
+      <c r="H24" s="3">
+        <v>11.107</v>
+      </c>
+      <c r="I24" s="3">
+        <v>3.577</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B25" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C25" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D25" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F25" s="3">
+        <v>89.103</v>
+      </c>
+      <c r="G25" s="3">
+        <v>12.318</v>
+      </c>
+      <c r="H25" s="3">
+        <v>11.568</v>
+      </c>
+      <c r="I25" s="3">
+        <v>3.765</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B26" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C26" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D26" s="3">
+        <v>1.98</v>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F26" s="3">
+        <v>88.07</v>
+      </c>
+      <c r="G26" s="3">
+        <v>13.267</v>
+      </c>
+      <c r="H26" s="3">
+        <v>12.039</v>
+      </c>
+      <c r="I26" s="3">
+        <v>3.873</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B27" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C27" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D27" s="3">
+        <v>1.96</v>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F27" s="3">
+        <v>86.365</v>
+      </c>
+      <c r="G27" s="3">
+        <v>14.467</v>
+      </c>
+      <c r="H27" s="3">
+        <v>12.508</v>
+      </c>
+      <c r="I27" s="3">
+        <v>3.881</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B28" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C28" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D28" s="3">
+        <v>2.02</v>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F28" s="3">
+        <v>81.889</v>
+      </c>
+      <c r="G28" s="3">
+        <v>12.003</v>
+      </c>
+      <c r="H28" s="3">
+        <v>13.912</v>
+      </c>
+      <c r="I28" s="3">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B29" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C29" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D29" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F29" s="3">
+        <v>81.46</v>
+      </c>
+      <c r="G29" s="3">
+        <v>12.621</v>
+      </c>
+      <c r="H29" s="3">
+        <v>14.281</v>
+      </c>
+      <c r="I29" s="3">
+        <v>3.575</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B30" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C30" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D30" s="3">
+        <v>1.98</v>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F30" s="3">
+        <v>80.344</v>
+      </c>
+      <c r="G30" s="3">
+        <v>13.428</v>
+      </c>
+      <c r="H30" s="3">
+        <v>14.677</v>
+      </c>
+      <c r="I30" s="3">
+        <v>3.58</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B31" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C31" s="3">
+        <v>1.48</v>
+      </c>
+      <c r="D31" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F31" s="3">
+        <v>80.124</v>
+      </c>
+      <c r="G31" s="3">
+        <v>5.163</v>
+      </c>
+      <c r="H31" s="3">
+        <v>23.88</v>
+      </c>
+      <c r="I31" s="3">
+        <v>2.571</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="B32" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C32" s="3">
+        <v>1.46</v>
+      </c>
+      <c r="D32" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F32" s="3">
+        <v>80.079</v>
+      </c>
+      <c r="G32" s="3">
+        <v>5.427</v>
+      </c>
+      <c r="H32" s="3">
+        <v>24.134</v>
+      </c>
+      <c r="I32" s="3">
+        <v>2.487</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B33" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C33" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D33" s="3">
+        <v>2.14</v>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F33" s="3">
+        <v>102.406</v>
+      </c>
+      <c r="G33" s="3">
+        <v>4.432</v>
+      </c>
+      <c r="H33" s="3">
+        <v>4.881</v>
+      </c>
+      <c r="I33" s="3">
+        <v>1.789</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B34" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C34" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D34" s="3">
+        <v>2.14</v>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F34" s="3">
+        <v>102.538</v>
+      </c>
+      <c r="G34" s="3">
+        <v>4.653</v>
+      </c>
+      <c r="H34" s="3">
+        <v>4.886</v>
+      </c>
+      <c r="I34" s="3">
+        <v>1.727</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B35" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C35" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D35" s="3">
+        <v>2.14</v>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F35" s="3">
+        <v>102.532</v>
+      </c>
+      <c r="G35" s="3">
+        <v>4.723</v>
+      </c>
+      <c r="H35" s="3">
+        <v>4.911</v>
+      </c>
+      <c r="I35" s="3">
+        <v>1.678</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B36" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C36" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D36" s="3">
+        <v>2.14</v>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F36" s="3">
+        <v>102.043</v>
+      </c>
+      <c r="G36" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="H36" s="3">
+        <v>4.915</v>
+      </c>
+      <c r="I36" s="3">
+        <v>1.859</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B37" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C37" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D37" s="3">
+        <v>2.14</v>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F37" s="3">
+        <v>102.449</v>
+      </c>
+      <c r="G37" s="3">
+        <v>4.712</v>
+      </c>
+      <c r="H37" s="3">
+        <v>4.945</v>
+      </c>
+      <c r="I37" s="3">
+        <v>1.651</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B38" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C38" s="3">
+        <v>1.14</v>
+      </c>
+      <c r="D38" s="3">
+        <v>2.16</v>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F38" s="3">
+        <v>99.496</v>
+      </c>
+      <c r="G38" s="3">
+        <v>2.405</v>
+      </c>
+      <c r="H38" s="3">
+        <v>4.973</v>
+      </c>
+      <c r="I38" s="3">
+        <v>1.672</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B39" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C39" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D39" s="3">
+        <v>2.22</v>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F39" s="3">
+        <v>98.986</v>
+      </c>
+      <c r="G39" s="3">
+        <v>2.93</v>
+      </c>
+      <c r="H39" s="3">
+        <v>5.036</v>
+      </c>
+      <c r="I39" s="3">
+        <v>1.676</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B40" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C40" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D40" s="3">
+        <v>2.22</v>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F40" s="3">
+        <v>98.974</v>
+      </c>
+      <c r="G40" s="3">
+        <v>2.82</v>
+      </c>
+      <c r="H40" s="3">
+        <v>5.066</v>
+      </c>
+      <c r="I40" s="3">
+        <v>1.719</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B41" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C41" s="3">
+        <v>1.28</v>
+      </c>
+      <c r="D41" s="3">
+        <v>2.38</v>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F41" s="3">
+        <v>93.221</v>
+      </c>
+      <c r="G41" s="3">
+        <v>1.985</v>
+      </c>
+      <c r="H41" s="3">
+        <v>5.074</v>
+      </c>
+      <c r="I41" s="3">
+        <v>1.306</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B42" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C42" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D42" s="3">
+        <v>2.22</v>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F42" s="3">
+        <v>98.962</v>
+      </c>
+      <c r="G42" s="3">
+        <v>2.731</v>
+      </c>
+      <c r="H42" s="3">
+        <v>5.076</v>
+      </c>
+      <c r="I42" s="3">
+        <v>1.756</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B43" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C43" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="D43" s="3">
+        <v>2.24</v>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F43" s="3">
+        <v>98.126</v>
+      </c>
+      <c r="G43" s="3">
+        <v>2.591</v>
+      </c>
+      <c r="H43" s="3">
+        <v>5.092</v>
+      </c>
+      <c r="I43" s="3">
+        <v>1.672</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B44" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C44" s="3">
+        <v>1.26</v>
+      </c>
+      <c r="D44" s="3">
+        <v>2.38</v>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F44" s="3">
+        <v>93.413</v>
+      </c>
+      <c r="G44" s="3">
+        <v>2.089</v>
+      </c>
+      <c r="H44" s="3">
+        <v>5.099</v>
+      </c>
+      <c r="I44" s="3">
+        <v>1.355</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B45" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C45" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D45" s="3">
+        <v>2.12</v>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F45" s="3">
+        <v>102.803</v>
+      </c>
+      <c r="G45" s="3">
+        <v>4.622</v>
+      </c>
+      <c r="H45" s="3">
+        <v>5.109</v>
+      </c>
+      <c r="I45" s="3">
+        <v>2.065</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B46" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C46" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D46" s="3">
+        <v>2.24</v>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F46" s="3">
+        <v>98.155</v>
+      </c>
+      <c r="G46" s="3">
+        <v>2.498</v>
+      </c>
+      <c r="H46" s="3">
+        <v>5.121</v>
+      </c>
+      <c r="I46" s="3">
+        <v>1.712</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B47" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C47" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D47" s="3">
+        <v>2.24</v>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F47" s="3">
+        <v>98.183</v>
+      </c>
+      <c r="G47" s="3">
+        <v>2.412</v>
+      </c>
+      <c r="H47" s="3">
+        <v>5.126</v>
+      </c>
+      <c r="I47" s="3">
+        <v>1.742</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B48" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C48" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="D48" s="3">
+        <v>2.26</v>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F48" s="3">
+        <v>97.363</v>
+      </c>
+      <c r="G48" s="3">
+        <v>2.301</v>
+      </c>
+      <c r="H48" s="3">
+        <v>5.151</v>
+      </c>
+      <c r="I48" s="3">
+        <v>1.688</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B49" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C49" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D49" s="3">
+        <v>2.26</v>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F49" s="3">
+        <v>97.428</v>
+      </c>
+      <c r="G49" s="3">
+        <v>2.199</v>
+      </c>
+      <c r="H49" s="3">
+        <v>5.153</v>
+      </c>
+      <c r="I49" s="3">
+        <v>1.709</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B50" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C50" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="D50" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F50" s="3">
+        <v>92.716</v>
+      </c>
+      <c r="G50" s="3">
+        <v>2.032</v>
+      </c>
+      <c r="H50" s="3">
+        <v>5.172</v>
+      </c>
+      <c r="I50" s="3">
+        <v>1.302</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B51" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C51" s="3">
+        <v>1.28</v>
+      </c>
+      <c r="D51" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F51" s="3">
+        <v>92.936</v>
+      </c>
+      <c r="G51" s="3">
+        <v>2.063</v>
+      </c>
+      <c r="H51" s="3">
+        <v>5.177</v>
+      </c>
+      <c r="I51" s="3">
+        <v>1.339</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B52" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C52" s="3">
+        <v>1.18</v>
+      </c>
+      <c r="D52" s="3">
+        <v>2.18</v>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F52" s="3">
+        <v>96.507</v>
+      </c>
+      <c r="G52" s="3">
+        <v>2.115</v>
+      </c>
+      <c r="H52" s="3">
+        <v>5.237</v>
+      </c>
+      <c r="I52" s="3">
+        <v>1.513</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B53" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C53" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="D53" s="3">
+        <v>2.42</v>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F53" s="3">
+        <v>92.471</v>
+      </c>
+      <c r="G53" s="3">
+        <v>2.083</v>
+      </c>
+      <c r="H53" s="3">
+        <v>5.274</v>
+      </c>
+      <c r="I53" s="3">
+        <v>1.332</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B54" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C54" s="3">
+        <v>1.32</v>
+      </c>
+      <c r="D54" s="3">
+        <v>2.42</v>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F54" s="3">
+        <v>92.22</v>
+      </c>
+      <c r="G54" s="3">
+        <v>2.118</v>
+      </c>
+      <c r="H54" s="3">
+        <v>5.283</v>
+      </c>
+      <c r="I54" s="3">
+        <v>1.317</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B55" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C55" s="3">
+        <v>1.32</v>
+      </c>
+      <c r="D55" s="3">
+        <v>2.44</v>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F55" s="3">
+        <v>92.013</v>
+      </c>
+      <c r="G55" s="3">
+        <v>2.146</v>
+      </c>
+      <c r="H55" s="3">
+        <v>5.385</v>
+      </c>
+      <c r="I55" s="3">
+        <v>1.337</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9">
+      <c r="A56" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B56" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C56" s="3">
+        <v>1.16</v>
+      </c>
+      <c r="D56" s="3">
+        <v>2.16</v>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F56" s="3">
+        <v>97.335</v>
+      </c>
+      <c r="G56" s="3">
+        <v>2.349</v>
+      </c>
+      <c r="H56" s="3">
+        <v>5.536</v>
+      </c>
+      <c r="I56" s="3">
+        <v>1.826</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9">
+      <c r="A57" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B57" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C57" s="3">
+        <v>1.18</v>
+      </c>
+      <c r="D57" s="3">
+        <v>2.16</v>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F57" s="3">
+        <v>93.542</v>
+      </c>
+      <c r="G57" s="3">
+        <v>3.813</v>
+      </c>
+      <c r="H57" s="3">
+        <v>6.703</v>
+      </c>
+      <c r="I57" s="3">
+        <v>2.202</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B58" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C58" s="3">
+        <v>1.14</v>
+      </c>
+      <c r="D58" s="3">
+        <v>2.12</v>
+      </c>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F58" s="3">
+        <v>94.198</v>
+      </c>
+      <c r="G58" s="3">
+        <v>6.64</v>
+      </c>
+      <c r="H58" s="3">
+        <v>7.505</v>
+      </c>
+      <c r="I58" s="3">
+        <v>2.993</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9">
+      <c r="A59" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B59" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C59" s="3">
+        <v>1.12</v>
+      </c>
+      <c r="D59" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F59" s="3">
+        <v>94.379</v>
+      </c>
+      <c r="G59" s="3">
+        <v>7.992</v>
+      </c>
+      <c r="H59" s="3">
+        <v>7.816</v>
+      </c>
+      <c r="I59" s="3">
+        <v>3.171</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B60" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C60" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="D60" s="3">
+        <v>2.08</v>
+      </c>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F60" s="3">
+        <v>94.556</v>
+      </c>
+      <c r="G60" s="3">
+        <v>8.94</v>
+      </c>
+      <c r="H60" s="3">
+        <v>8.089</v>
+      </c>
+      <c r="I60" s="3">
+        <v>3.221</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9">
+      <c r="A61" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B61" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C61" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D61" s="3">
+        <v>2.06</v>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F61" s="3">
+        <v>94.609</v>
+      </c>
+      <c r="G61" s="3">
+        <v>9.697</v>
+      </c>
+      <c r="H61" s="3">
+        <v>8.382</v>
+      </c>
+      <c r="I61" s="3">
+        <v>3.252</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9">
+      <c r="A62" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B62" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C62" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D62" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F62" s="3">
+        <v>96.57</v>
+      </c>
+      <c r="G62" s="3">
+        <v>10.914</v>
+      </c>
+      <c r="H62" s="3">
+        <v>8.412</v>
+      </c>
+      <c r="I62" s="3">
+        <v>3.755</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9">
+      <c r="A63" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B63" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C63" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D63" s="3">
+        <v>2.04</v>
+      </c>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F63" s="3">
+        <v>94.494</v>
+      </c>
+      <c r="G63" s="3">
+        <v>10.343</v>
+      </c>
+      <c r="H63" s="3">
+        <v>8.74</v>
+      </c>
+      <c r="I63" s="3">
+        <v>3.355</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9">
+      <c r="A64" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B64" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C64" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="D64" s="3">
+        <v>2.16</v>
+      </c>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F64" s="3">
+        <v>87.103</v>
+      </c>
+      <c r="G64" s="3">
+        <v>6.257</v>
+      </c>
+      <c r="H64" s="3">
+        <v>8.837</v>
+      </c>
+      <c r="I64" s="3">
+        <v>2.828</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9">
+      <c r="A65" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B65" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C65" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D65" s="3">
+        <v>2.02</v>
+      </c>
+      <c r="E65" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F65" s="3">
+        <v>94.233</v>
+      </c>
+      <c r="G65" s="3">
+        <v>10.899</v>
+      </c>
+      <c r="H65" s="3">
+        <v>9.176</v>
+      </c>
+      <c r="I65" s="3">
+        <v>3.555</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9">
+      <c r="A66" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B66" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C66" s="3">
+        <v>1.18</v>
+      </c>
+      <c r="D66" s="3">
+        <v>2.14</v>
+      </c>
+      <c r="E66" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F66" s="3">
+        <v>87.867</v>
+      </c>
+      <c r="G66" s="3">
+        <v>7.122</v>
+      </c>
+      <c r="H66" s="3">
+        <v>9.226</v>
+      </c>
+      <c r="I66" s="3">
+        <v>3.065</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9">
+      <c r="A67" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B67" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C67" s="3">
+        <v>1.16</v>
+      </c>
+      <c r="D67" s="3">
+        <v>2.12</v>
+      </c>
+      <c r="E67" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F67" s="3">
+        <v>88.494</v>
+      </c>
+      <c r="G67" s="3">
+        <v>8.147</v>
+      </c>
+      <c r="H67" s="3">
+        <v>9.553</v>
+      </c>
+      <c r="I67" s="3">
+        <v>3.207</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9">
+      <c r="A68" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B68" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C68" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D68" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="E68" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F68" s="3">
+        <v>93.759</v>
+      </c>
+      <c r="G68" s="3">
+        <v>11.553</v>
+      </c>
+      <c r="H68" s="3">
+        <v>9.669</v>
+      </c>
+      <c r="I68" s="3">
+        <v>3.797</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9">
+      <c r="A69" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B69" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C69" s="3">
+        <v>1.14</v>
+      </c>
+      <c r="D69" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="E69" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F69" s="3">
+        <v>89.067</v>
+      </c>
+      <c r="G69" s="3">
+        <v>9.004</v>
+      </c>
+      <c r="H69" s="3">
+        <v>9.821</v>
+      </c>
+      <c r="I69" s="3">
+        <v>3.237</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9">
+      <c r="A70" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B70" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C70" s="3">
+        <v>1.12</v>
+      </c>
+      <c r="D70" s="3">
+        <v>2.08</v>
+      </c>
+      <c r="E70" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F70" s="3">
+        <v>89.517</v>
+      </c>
+      <c r="G70" s="3">
+        <v>9.721</v>
+      </c>
+      <c r="H70" s="3">
+        <v>10.073</v>
+      </c>
+      <c r="I70" s="3">
+        <v>3.23</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9">
+      <c r="A71" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B71" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C71" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D71" s="3">
+        <v>1.98</v>
+      </c>
+      <c r="E71" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F71" s="3">
+        <v>92.876</v>
+      </c>
+      <c r="G71" s="3">
+        <v>12.519</v>
+      </c>
+      <c r="H71" s="3">
+        <v>10.167</v>
+      </c>
+      <c r="I71" s="3">
+        <v>3.986</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9">
+      <c r="A72" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B72" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C72" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="D72" s="3">
+        <v>2.06</v>
+      </c>
+      <c r="E72" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F72" s="3">
+        <v>89.757</v>
+      </c>
+      <c r="G72" s="3">
+        <v>10.396</v>
+      </c>
+      <c r="H72" s="3">
+        <v>10.355</v>
+      </c>
+      <c r="I72" s="3">
+        <v>3.267</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9">
+      <c r="A73" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B73" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C73" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D73" s="3">
+        <v>2.04</v>
+      </c>
+      <c r="E73" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F73" s="3">
+        <v>89.78</v>
+      </c>
+      <c r="G73" s="3">
+        <v>11.024</v>
+      </c>
+      <c r="H73" s="3">
+        <v>10.696</v>
+      </c>
+      <c r="I73" s="3">
+        <v>3.389</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9">
+      <c r="A74" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B74" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C74" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D74" s="3">
+        <v>2.02</v>
+      </c>
+      <c r="E74" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F74" s="3">
+        <v>89.598</v>
+      </c>
+      <c r="G74" s="3">
+        <v>11.613</v>
+      </c>
+      <c r="H74" s="3">
+        <v>11.107</v>
+      </c>
+      <c r="I74" s="3">
+        <v>3.577</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9">
+      <c r="A75" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B75" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C75" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D75" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="E75" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F75" s="3">
+        <v>89.103</v>
+      </c>
+      <c r="G75" s="3">
+        <v>12.318</v>
+      </c>
+      <c r="H75" s="3">
+        <v>11.568</v>
+      </c>
+      <c r="I75" s="3">
+        <v>3.765</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9">
+      <c r="A76" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B76" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C76" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="D76" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E76" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F76" s="3">
+        <v>80.102</v>
+      </c>
+      <c r="G76" s="3">
+        <v>4.882</v>
+      </c>
+      <c r="H76" s="3">
+        <v>23.392</v>
+      </c>
+      <c r="I76" s="3">
+        <v>2.544</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9">
+      <c r="A77" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B77" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C77" s="3">
+        <v>1.48</v>
+      </c>
+      <c r="D77" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E77" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F77" s="3">
+        <v>80.124</v>
+      </c>
+      <c r="G77" s="3">
+        <v>5.163</v>
+      </c>
+      <c r="H77" s="3">
+        <v>23.88</v>
+      </c>
+      <c r="I77" s="3">
+        <v>2.571</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9">
+      <c r="A78" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B78" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C78" s="3">
+        <v>1.44</v>
+      </c>
+      <c r="D78" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E78" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F78" s="3">
+        <v>80.062</v>
+      </c>
+      <c r="G78" s="3">
+        <v>5.454</v>
+      </c>
+      <c r="H78" s="3">
+        <v>24.126</v>
+      </c>
+      <c r="I78" s="3">
+        <v>2.335</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9">
+      <c r="A79" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B79" s="3">
+        <v>0.841</v>
+      </c>
+      <c r="C79" s="3">
+        <v>1.46</v>
+      </c>
+      <c r="D79" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E79" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F79" s="3">
+        <v>80.079</v>
+      </c>
+      <c r="G79" s="3">
+        <v>5.427</v>
+      </c>
+      <c r="H79" s="3">
+        <v>24.134</v>
+      </c>
+      <c r="I79" s="3">
+        <v>2.487</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9">
+      <c r="A80" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B80" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C80" s="3">
+        <v>1.16</v>
+      </c>
+      <c r="D80" s="3">
+        <v>2.18</v>
+      </c>
+      <c r="E80" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F80" s="3">
+        <v>98.625</v>
+      </c>
+      <c r="G80" s="3">
+        <v>2.3</v>
+      </c>
+      <c r="H80" s="3">
+        <v>4.75</v>
+      </c>
+      <c r="I80" s="3">
+        <v>1.528</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9">
+      <c r="A81" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B81" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C81" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="D81" s="3">
+        <v>2.16</v>
+      </c>
+      <c r="E81" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F81" s="3">
+        <v>101.652</v>
+      </c>
+      <c r="G81" s="3">
+        <v>4.291</v>
+      </c>
+      <c r="H81" s="3">
+        <v>4.868</v>
+      </c>
+      <c r="I81" s="3">
+        <v>1.591</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9">
+      <c r="A82" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B82" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C82" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D82" s="3">
+        <v>2.16</v>
+      </c>
+      <c r="E82" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F82" s="3">
+        <v>101.54</v>
+      </c>
+      <c r="G82" s="3">
+        <v>4.203</v>
+      </c>
+      <c r="H82" s="3">
+        <v>4.907</v>
+      </c>
+      <c r="I82" s="3">
+        <v>1.615</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9">
+      <c r="A83" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B83" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C83" s="3">
+        <v>1.14</v>
+      </c>
+      <c r="D83" s="3">
+        <v>2.16</v>
+      </c>
+      <c r="E83" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F83" s="3">
+        <v>99.496</v>
+      </c>
+      <c r="G83" s="3">
+        <v>2.405</v>
+      </c>
+      <c r="H83" s="3">
+        <v>4.973</v>
+      </c>
+      <c r="I83" s="3">
+        <v>1.672</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9">
+      <c r="A84" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B84" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C84" s="3">
+        <v>1.26</v>
+      </c>
+      <c r="D84" s="3">
+        <v>2.36</v>
+      </c>
+      <c r="E84" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F84" s="3">
+        <v>93.743</v>
+      </c>
+      <c r="G84" s="3">
+        <v>1.987</v>
+      </c>
+      <c r="H84" s="3">
+        <v>4.995</v>
+      </c>
+      <c r="I84" s="3">
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9">
+      <c r="A85" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B85" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C85" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="D85" s="3">
+        <v>2.14</v>
+      </c>
+      <c r="E85" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F85" s="3">
+        <v>101.311</v>
+      </c>
+      <c r="G85" s="3">
+        <v>3.337</v>
+      </c>
+      <c r="H85" s="3">
+        <v>5.027</v>
+      </c>
+      <c r="I85" s="3">
+        <v>1.949</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9">
+      <c r="A86" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B86" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C86" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D86" s="3">
+        <v>2.22</v>
+      </c>
+      <c r="E86" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F86" s="3">
+        <v>98.986</v>
+      </c>
+      <c r="G86" s="3">
+        <v>2.93</v>
+      </c>
+      <c r="H86" s="3">
+        <v>5.036</v>
+      </c>
+      <c r="I86" s="3">
+        <v>1.676</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9">
+      <c r="A87" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B87" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C87" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="D87" s="3">
+        <v>2.3</v>
+      </c>
+      <c r="E87" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F87" s="3">
+        <v>96.467</v>
+      </c>
+      <c r="G87" s="3">
+        <v>1.767</v>
+      </c>
+      <c r="H87" s="3">
+        <v>5.067</v>
+      </c>
+      <c r="I87" s="3">
+        <v>1.622</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9">
+      <c r="A88" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B88" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C88" s="3">
+        <v>1.28</v>
+      </c>
+      <c r="D88" s="3">
+        <v>2.38</v>
+      </c>
+      <c r="E88" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F88" s="3">
+        <v>93.221</v>
+      </c>
+      <c r="G88" s="3">
+        <v>1.985</v>
+      </c>
+      <c r="H88" s="3">
+        <v>5.074</v>
+      </c>
+      <c r="I88" s="3">
+        <v>1.306</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9">
+      <c r="A89" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B89" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C89" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="D89" s="3">
+        <v>2.24</v>
+      </c>
+      <c r="E89" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F89" s="3">
+        <v>98.126</v>
+      </c>
+      <c r="G89" s="3">
+        <v>2.591</v>
+      </c>
+      <c r="H89" s="3">
+        <v>5.092</v>
+      </c>
+      <c r="I89" s="3">
+        <v>1.672</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9">
+      <c r="A90" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B90" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C90" s="3">
+        <v>1.26</v>
+      </c>
+      <c r="D90" s="3">
+        <v>2.38</v>
+      </c>
+      <c r="E90" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F90" s="3">
+        <v>93.413</v>
+      </c>
+      <c r="G90" s="3">
+        <v>2.089</v>
+      </c>
+      <c r="H90" s="3">
+        <v>5.099</v>
+      </c>
+      <c r="I90" s="3">
+        <v>1.355</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9">
+      <c r="A91" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B91" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C91" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D91" s="3">
+        <v>2.24</v>
+      </c>
+      <c r="E91" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F91" s="3">
+        <v>98.155</v>
+      </c>
+      <c r="G91" s="3">
+        <v>2.498</v>
+      </c>
+      <c r="H91" s="3">
+        <v>5.121</v>
+      </c>
+      <c r="I91" s="3">
+        <v>1.712</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9">
+      <c r="A92" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B92" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C92" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D92" s="3">
+        <v>2.28</v>
+      </c>
+      <c r="E92" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F92" s="3">
+        <v>96.89</v>
+      </c>
+      <c r="G92" s="3">
+        <v>1.91</v>
+      </c>
+      <c r="H92" s="3">
+        <v>5.125</v>
+      </c>
+      <c r="I92" s="3">
+        <v>1.678</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9">
+      <c r="A93" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B93" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C93" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="D93" s="3">
+        <v>2.24</v>
+      </c>
+      <c r="E93" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F93" s="3">
+        <v>98.183</v>
+      </c>
+      <c r="G93" s="3">
+        <v>2.412</v>
+      </c>
+      <c r="H93" s="3">
+        <v>5.126</v>
+      </c>
+      <c r="I93" s="3">
+        <v>1.742</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9">
+      <c r="A94" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B94" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C94" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="D94" s="3">
+        <v>2.26</v>
+      </c>
+      <c r="E94" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F94" s="3">
+        <v>97.363</v>
+      </c>
+      <c r="G94" s="3">
+        <v>2.301</v>
+      </c>
+      <c r="H94" s="3">
+        <v>5.151</v>
+      </c>
+      <c r="I94" s="3">
+        <v>1.688</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9">
+      <c r="A95" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B95" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C95" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="D95" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="E95" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F95" s="3">
+        <v>92.716</v>
+      </c>
+      <c r="G95" s="3">
+        <v>2.032</v>
+      </c>
+      <c r="H95" s="3">
+        <v>5.172</v>
+      </c>
+      <c r="I95" s="3">
+        <v>1.302</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9">
+      <c r="A96" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B96" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C96" s="3">
+        <v>1.28</v>
+      </c>
+      <c r="D96" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="E96" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F96" s="3">
+        <v>92.936</v>
+      </c>
+      <c r="G96" s="3">
+        <v>2.063</v>
+      </c>
+      <c r="H96" s="3">
+        <v>5.177</v>
+      </c>
+      <c r="I96" s="3">
+        <v>1.339</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9">
+      <c r="A97" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B97" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C97" s="3">
+        <v>1.18</v>
+      </c>
+      <c r="D97" s="3">
+        <v>2.18</v>
+      </c>
+      <c r="E97" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F97" s="3">
+        <v>96.507</v>
+      </c>
+      <c r="G97" s="3">
+        <v>2.115</v>
+      </c>
+      <c r="H97" s="3">
+        <v>5.237</v>
+      </c>
+      <c r="I97" s="3">
+        <v>1.513</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9">
+      <c r="A98" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B98" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C98" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="D98" s="3">
+        <v>2.42</v>
+      </c>
+      <c r="E98" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F98" s="3">
+        <v>92.471</v>
+      </c>
+      <c r="G98" s="3">
+        <v>2.083</v>
+      </c>
+      <c r="H98" s="3">
+        <v>5.274</v>
+      </c>
+      <c r="I98" s="3">
+        <v>1.332</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9">
+      <c r="A99" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B99" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C99" s="3">
+        <v>1.32</v>
+      </c>
+      <c r="D99" s="3">
+        <v>2.42</v>
+      </c>
+      <c r="E99" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F99" s="3">
+        <v>92.22</v>
+      </c>
+      <c r="G99" s="3">
+        <v>2.118</v>
+      </c>
+      <c r="H99" s="3">
+        <v>5.283</v>
+      </c>
+      <c r="I99" s="3">
+        <v>1.317</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9">
+      <c r="A100" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B100" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C100" s="3">
+        <v>1.32</v>
+      </c>
+      <c r="D100" s="3">
+        <v>2.44</v>
+      </c>
+      <c r="E100" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F100" s="3">
+        <v>92.013</v>
+      </c>
+      <c r="G100" s="3">
+        <v>2.146</v>
+      </c>
+      <c r="H100" s="3">
+        <v>5.385</v>
+      </c>
+      <c r="I100" s="3">
+        <v>1.337</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9">
+      <c r="A101" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B101" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C101" s="3">
+        <v>1.34</v>
+      </c>
+      <c r="D101" s="3">
+        <v>2.46</v>
+      </c>
+      <c r="E101" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F101" s="3">
+        <v>91.56</v>
+      </c>
+      <c r="G101" s="3">
+        <v>2.237</v>
+      </c>
+      <c r="H101" s="3">
+        <v>5.504</v>
+      </c>
+      <c r="I101" s="3">
+        <v>1.363</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9">
+      <c r="A102" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B102" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C102" s="3">
+        <v>1.16</v>
+      </c>
+      <c r="D102" s="3">
+        <v>2.16</v>
+      </c>
+      <c r="E102" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F102" s="3">
+        <v>97.335</v>
+      </c>
+      <c r="G102" s="3">
+        <v>2.349</v>
+      </c>
+      <c r="H102" s="3">
+        <v>5.536</v>
+      </c>
+      <c r="I102" s="3">
+        <v>1.826</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9">
+      <c r="A103" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B103" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C103" s="3">
+        <v>1.36</v>
+      </c>
+      <c r="D103" s="3">
+        <v>2.48</v>
+      </c>
+      <c r="E103" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F103" s="3">
+        <v>91.111</v>
+      </c>
+      <c r="G103" s="3">
+        <v>2.343</v>
+      </c>
+      <c r="H103" s="3">
+        <v>5.629</v>
+      </c>
+      <c r="I103" s="3">
+        <v>1.411</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9">
+      <c r="A104" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B104" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C104" s="3">
+        <v>1.34</v>
+      </c>
+      <c r="D104" s="3">
+        <v>2.34</v>
+      </c>
+      <c r="E104" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F104" s="3">
+        <v>88.21</v>
+      </c>
+      <c r="G104" s="3">
+        <v>2.803</v>
+      </c>
+      <c r="H104" s="3">
+        <v>5.657</v>
+      </c>
+      <c r="I104" s="3">
+        <v>1.376</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9">
+      <c r="A105" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B105" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C105" s="3">
+        <v>1.38</v>
+      </c>
+      <c r="D105" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="E105" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F105" s="3">
+        <v>90.665</v>
+      </c>
+      <c r="G105" s="3">
+        <v>2.458</v>
+      </c>
+      <c r="H105" s="3">
+        <v>5.756</v>
+      </c>
+      <c r="I105" s="3">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9">
+      <c r="A106" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B106" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C106" s="3">
+        <v>1.36</v>
+      </c>
+      <c r="D106" s="3">
+        <v>2.36</v>
+      </c>
+      <c r="E106" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F106" s="3">
+        <v>87.191</v>
+      </c>
+      <c r="G106" s="3">
+        <v>2.766</v>
+      </c>
+      <c r="H106" s="3">
+        <v>5.81</v>
+      </c>
+      <c r="I106" s="3">
+        <v>1.395</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9">
+      <c r="A107" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B107" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C107" s="3">
+        <v>1.38</v>
+      </c>
+      <c r="D107" s="3">
+        <v>2.38</v>
+      </c>
+      <c r="E107" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F107" s="3">
+        <v>86.138</v>
+      </c>
+      <c r="G107" s="3">
+        <v>2.701</v>
+      </c>
+      <c r="H107" s="3">
+        <v>5.936</v>
+      </c>
+      <c r="I107" s="3">
+        <v>1.409</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9">
+      <c r="A108" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B108" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C108" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="D108" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="E108" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F108" s="3">
+        <v>85.025</v>
+      </c>
+      <c r="G108" s="3">
+        <v>2.632</v>
+      </c>
+      <c r="H108" s="3">
+        <v>6.03</v>
+      </c>
+      <c r="I108" s="3">
+        <v>1.444</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9">
+      <c r="A109" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B109" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C109" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="D109" s="3">
+        <v>2.16</v>
+      </c>
+      <c r="E109" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F109" s="3">
+        <v>87.103</v>
+      </c>
+      <c r="G109" s="3">
+        <v>6.257</v>
+      </c>
+      <c r="H109" s="3">
+        <v>8.837</v>
+      </c>
+      <c r="I109" s="3">
+        <v>2.828</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9">
+      <c r="A110" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B110" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C110" s="3">
+        <v>1.16</v>
+      </c>
+      <c r="D110" s="3">
+        <v>2.12</v>
+      </c>
+      <c r="E110" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F110" s="3">
+        <v>88.494</v>
+      </c>
+      <c r="G110" s="3">
+        <v>8.147</v>
+      </c>
+      <c r="H110" s="3">
+        <v>9.553</v>
+      </c>
+      <c r="I110" s="3">
+        <v>3.207</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9">
+      <c r="A111" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B111" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C111" s="3">
+        <v>1.14</v>
+      </c>
+      <c r="D111" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="E111" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F111" s="3">
+        <v>89.067</v>
+      </c>
+      <c r="G111" s="3">
+        <v>9.004</v>
+      </c>
+      <c r="H111" s="3">
+        <v>9.821</v>
+      </c>
+      <c r="I111" s="3">
+        <v>3.237</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9">
+      <c r="A112" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B112" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C112" s="3">
+        <v>1.12</v>
+      </c>
+      <c r="D112" s="3">
+        <v>2.08</v>
+      </c>
+      <c r="E112" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F112" s="3">
+        <v>89.517</v>
+      </c>
+      <c r="G112" s="3">
+        <v>9.721</v>
+      </c>
+      <c r="H112" s="3">
+        <v>10.073</v>
+      </c>
+      <c r="I112" s="3">
+        <v>3.23</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9">
+      <c r="A113" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B113" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C113" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="D113" s="3">
+        <v>2.06</v>
+      </c>
+      <c r="E113" s="1" t="inlineStr">
+        <is>
+          <t>Y-dominant</t>
+        </is>
+      </c>
+      <c r="F113" s="3">
+        <v>89.757</v>
+      </c>
+      <c r="G113" s="3">
+        <v>10.396</v>
+      </c>
+      <c r="H113" s="3">
+        <v>10.355</v>
+      </c>
+      <c r="I113" s="3">
+        <v>3.267</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9">
+      <c r="A114" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B114" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C114" s="3">
+        <v>1.52</v>
+      </c>
+      <c r="D114" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E114" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F114" s="3">
+        <v>79.873</v>
+      </c>
+      <c r="G114" s="3">
+        <v>4.707</v>
+      </c>
+      <c r="H114" s="3">
+        <v>22.687</v>
+      </c>
+      <c r="I114" s="3">
+        <v>2.419</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9">
+      <c r="A115" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B115" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C115" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="D115" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E115" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F115" s="3">
+        <v>80.102</v>
+      </c>
+      <c r="G115" s="3">
+        <v>4.882</v>
+      </c>
+      <c r="H115" s="3">
+        <v>23.392</v>
+      </c>
+      <c r="I115" s="3">
+        <v>2.544</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9">
+      <c r="A116" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B116" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C116" s="3">
+        <v>1.48</v>
+      </c>
+      <c r="D116" s="3">
+        <v>1.06</v>
+      </c>
+      <c r="E116" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F116" s="3">
+        <v>77.433</v>
+      </c>
+      <c r="G116" s="3">
+        <v>4.446</v>
+      </c>
+      <c r="H116" s="3">
+        <v>23.683</v>
+      </c>
+      <c r="I116" s="3">
+        <v>2.035</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9">
+      <c r="A117" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B117" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C117" s="3">
+        <v>1.46</v>
+      </c>
+      <c r="D117" s="3">
+        <v>1.04</v>
+      </c>
+      <c r="E117" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F117" s="3">
+        <v>78.398</v>
+      </c>
+      <c r="G117" s="3">
+        <v>4.78</v>
+      </c>
+      <c r="H117" s="3">
+        <v>23.759</v>
+      </c>
+      <c r="I117" s="3">
+        <v>2.097</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9">
+      <c r="A118" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B118" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C118" s="3">
+        <v>1.48</v>
+      </c>
+      <c r="D118" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E118" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F118" s="3">
+        <v>80.124</v>
+      </c>
+      <c r="G118" s="3">
+        <v>5.163</v>
+      </c>
+      <c r="H118" s="3">
+        <v>23.88</v>
+      </c>
+      <c r="I118" s="3">
+        <v>2.571</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9">
+      <c r="A119" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B119" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C119" s="3">
+        <v>1.46</v>
+      </c>
+      <c r="D119" s="3">
+        <v>1.02</v>
+      </c>
+      <c r="E119" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F119" s="3">
+        <v>79.273</v>
+      </c>
+      <c r="G119" s="3">
+        <v>5.164</v>
+      </c>
+      <c r="H119" s="3">
+        <v>24.036</v>
+      </c>
+      <c r="I119" s="3">
+        <v>2.276</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9">
+      <c r="A120" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B120" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C120" s="3">
+        <v>1.44</v>
+      </c>
+      <c r="D120" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E120" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F120" s="3">
+        <v>80.062</v>
+      </c>
+      <c r="G120" s="3">
+        <v>5.454</v>
+      </c>
+      <c r="H120" s="3">
+        <v>24.126</v>
+      </c>
+      <c r="I120" s="3">
+        <v>2.335</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9">
+      <c r="A121" s="1">
+        <v>1.645</v>
+      </c>
+      <c r="B121" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C121" s="3">
+        <v>1.46</v>
+      </c>
+      <c r="D121" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E121" s="1" t="inlineStr">
+        <is>
+          <t>Bar-dominant</t>
+        </is>
+      </c>
+      <c r="F121" s="3">
+        <v>80.079</v>
+      </c>
+      <c r="G121" s="3">
+        <v>5.427</v>
+      </c>
+      <c r="H121" s="3">
+        <v>24.134</v>
+      </c>
+      <c r="I121" s="3">
+        <v>2.487</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>